<commit_message>
fix: harden OGC API Features review gaps
</commit_message>
<xml_diff>
--- a/demo/data/clinic_capacity.xlsx
+++ b/demo/data/clinic_capacity.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,10 +461,20 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>map_latitude</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>map_longitude</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>exact_latitude</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>exact_longitude</t>
         </is>
@@ -512,9 +522,15 @@
         </is>
       </c>
       <c r="I2" t="n">
+        <v>16.7179</v>
+      </c>
+      <c r="J2" t="n">
+        <v>42.9685</v>
+      </c>
+      <c r="K2" t="n">
         <v>17.0366</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>30.7467</v>
       </c>
     </row>
@@ -560,9 +576,15 @@
         </is>
       </c>
       <c r="I3" t="n">
+        <v>11.1337</v>
+      </c>
+      <c r="J3" t="n">
+        <v>38.9886</v>
+      </c>
+      <c r="K3" t="n">
         <v>10.5168</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>41.6004</v>
       </c>
     </row>
@@ -608,9 +630,15 @@
         </is>
       </c>
       <c r="I4" t="n">
+        <v>16.9008</v>
+      </c>
+      <c r="J4" t="n">
+        <v>43.3009</v>
+      </c>
+      <c r="K4" t="n">
         <v>14.9289</v>
       </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
         <v>35.7311</v>
       </c>
     </row>
@@ -656,9 +684,15 @@
         </is>
       </c>
       <c r="I5" t="n">
+        <v>8.1721</v>
+      </c>
+      <c r="J5" t="n">
+        <v>37.1329</v>
+      </c>
+      <c r="K5" t="n">
         <v>8.170500000000001</v>
       </c>
-      <c r="J5" t="n">
+      <c r="L5" t="n">
         <v>32.1891</v>
       </c>
     </row>
@@ -704,9 +738,15 @@
         </is>
       </c>
       <c r="I6" t="n">
+        <v>7.9808</v>
+      </c>
+      <c r="J6" t="n">
+        <v>37.2776</v>
+      </c>
+      <c r="K6" t="n">
         <v>9.377599999999999</v>
       </c>
-      <c r="J6" t="n">
+      <c r="L6" t="n">
         <v>43.0717</v>
       </c>
     </row>
@@ -752,9 +792,15 @@
         </is>
       </c>
       <c r="I7" t="n">
+        <v>16.7397</v>
+      </c>
+      <c r="J7" t="n">
+        <v>43.1806</v>
+      </c>
+      <c r="K7" t="n">
         <v>11.14</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>30.7817</v>
       </c>
     </row>
@@ -800,9 +846,15 @@
         </is>
       </c>
       <c r="I8" t="n">
+        <v>16.8778</v>
+      </c>
+      <c r="J8" t="n">
+        <v>43.0522</v>
+      </c>
+      <c r="K8" t="n">
         <v>10.0908</v>
       </c>
-      <c r="J8" t="n">
+      <c r="L8" t="n">
         <v>35.7141</v>
       </c>
     </row>
@@ -848,9 +900,15 @@
         </is>
       </c>
       <c r="I9" t="n">
+        <v>17.3162</v>
+      </c>
+      <c r="J9" t="n">
+        <v>43.2875</v>
+      </c>
+      <c r="K9" t="n">
         <v>10.0749</v>
       </c>
-      <c r="J9" t="n">
+      <c r="L9" t="n">
         <v>43.9549</v>
       </c>
     </row>
@@ -896,9 +954,15 @@
         </is>
       </c>
       <c r="I10" t="n">
+        <v>16.6889</v>
+      </c>
+      <c r="J10" t="n">
+        <v>43.3322</v>
+      </c>
+      <c r="K10" t="n">
         <v>0.8832</v>
       </c>
-      <c r="J10" t="n">
+      <c r="L10" t="n">
         <v>31.9181</v>
       </c>
     </row>
@@ -944,9 +1008,15 @@
         </is>
       </c>
       <c r="I11" t="n">
+        <v>17.1821</v>
+      </c>
+      <c r="J11" t="n">
+        <v>43.2414</v>
+      </c>
+      <c r="K11" t="n">
         <v>6.2602</v>
       </c>
-      <c r="J11" t="n">
+      <c r="L11" t="n">
         <v>43.3901</v>
       </c>
     </row>
@@ -992,9 +1062,15 @@
         </is>
       </c>
       <c r="I12" t="n">
+        <v>8.231199999999999</v>
+      </c>
+      <c r="J12" t="n">
+        <v>36.7632</v>
+      </c>
+      <c r="K12" t="n">
         <v>2.9724</v>
       </c>
-      <c r="J12" t="n">
+      <c r="L12" t="n">
         <v>33.4479</v>
       </c>
     </row>
@@ -1040,9 +1116,15 @@
         </is>
       </c>
       <c r="I13" t="n">
+        <v>5.2756</v>
+      </c>
+      <c r="J13" t="n">
+        <v>34.7054</v>
+      </c>
+      <c r="K13" t="n">
         <v>19.7764</v>
       </c>
-      <c r="J13" t="n">
+      <c r="L13" t="n">
         <v>38.4128</v>
       </c>
     </row>
@@ -1088,9 +1170,15 @@
         </is>
       </c>
       <c r="I14" t="n">
+        <v>7.9144</v>
+      </c>
+      <c r="J14" t="n">
+        <v>36.6888</v>
+      </c>
+      <c r="K14" t="n">
         <v>3.6131</v>
       </c>
-      <c r="J14" t="n">
+      <c r="L14" t="n">
         <v>32.5244</v>
       </c>
     </row>
@@ -1136,9 +1224,15 @@
         </is>
       </c>
       <c r="I15" t="n">
+        <v>10.956</v>
+      </c>
+      <c r="J15" t="n">
+        <v>38.7861</v>
+      </c>
+      <c r="K15" t="n">
         <v>18.4083</v>
       </c>
-      <c r="J15" t="n">
+      <c r="L15" t="n">
         <v>33.6924</v>
       </c>
     </row>
@@ -1184,9 +1278,15 @@
         </is>
       </c>
       <c r="I16" t="n">
+        <v>11.1077</v>
+      </c>
+      <c r="J16" t="n">
+        <v>38.8608</v>
+      </c>
+      <c r="K16" t="n">
         <v>11.8068</v>
       </c>
-      <c r="J16" t="n">
+      <c r="L16" t="n">
         <v>44.2683</v>
       </c>
     </row>
@@ -1232,9 +1332,15 @@
         </is>
       </c>
       <c r="I17" t="n">
+        <v>14.0552</v>
+      </c>
+      <c r="J17" t="n">
+        <v>41.2582</v>
+      </c>
+      <c r="K17" t="n">
         <v>19.104</v>
       </c>
-      <c r="J17" t="n">
+      <c r="L17" t="n">
         <v>38.9131</v>
       </c>
     </row>
@@ -1280,9 +1386,15 @@
         </is>
       </c>
       <c r="I18" t="n">
+        <v>4.8748</v>
+      </c>
+      <c r="J18" t="n">
+        <v>35.0946</v>
+      </c>
+      <c r="K18" t="n">
         <v>16.0312</v>
       </c>
-      <c r="J18" t="n">
+      <c r="L18" t="n">
         <v>34.2443</v>
       </c>
     </row>
@@ -1328,9 +1440,15 @@
         </is>
       </c>
       <c r="I19" t="n">
+        <v>13.7062</v>
+      </c>
+      <c r="J19" t="n">
+        <v>40.8526</v>
+      </c>
+      <c r="K19" t="n">
         <v>4.8016</v>
       </c>
-      <c r="J19" t="n">
+      <c r="L19" t="n">
         <v>41.5632</v>
       </c>
     </row>
@@ -1376,9 +1494,15 @@
         </is>
       </c>
       <c r="I20" t="n">
+        <v>7.7812</v>
+      </c>
+      <c r="J20" t="n">
+        <v>36.7382</v>
+      </c>
+      <c r="K20" t="n">
         <v>5.9709</v>
       </c>
-      <c r="J20" t="n">
+      <c r="L20" t="n">
         <v>42.0165</v>
       </c>
     </row>
@@ -1424,9 +1548,15 @@
         </is>
       </c>
       <c r="I21" t="n">
+        <v>14.1779</v>
+      </c>
+      <c r="J21" t="n">
+        <v>40.8197</v>
+      </c>
+      <c r="K21" t="n">
         <v>3.9974</v>
       </c>
-      <c r="J21" t="n">
+      <c r="L21" t="n">
         <v>36.6816</v>
       </c>
     </row>
@@ -1472,9 +1602,15 @@
         </is>
       </c>
       <c r="I22" t="n">
+        <v>7.7566</v>
+      </c>
+      <c r="J22" t="n">
+        <v>36.9243</v>
+      </c>
+      <c r="K22" t="n">
         <v>12.6137</v>
       </c>
-      <c r="J22" t="n">
+      <c r="L22" t="n">
         <v>31.3942</v>
       </c>
     </row>
@@ -1520,9 +1656,15 @@
         </is>
       </c>
       <c r="I23" t="n">
+        <v>10.9489</v>
+      </c>
+      <c r="J23" t="n">
+        <v>39.0805</v>
+      </c>
+      <c r="K23" t="n">
         <v>12.5912</v>
       </c>
-      <c r="J23" t="n">
+      <c r="L23" t="n">
         <v>37.8702</v>
       </c>
     </row>
@@ -1568,9 +1710,15 @@
         </is>
       </c>
       <c r="I24" t="n">
+        <v>7.9549</v>
+      </c>
+      <c r="J24" t="n">
+        <v>36.9245</v>
+      </c>
+      <c r="K24" t="n">
         <v>10.4618</v>
       </c>
-      <c r="J24" t="n">
+      <c r="L24" t="n">
         <v>34.4322</v>
       </c>
     </row>
@@ -1616,9 +1764,15 @@
         </is>
       </c>
       <c r="I25" t="n">
+        <v>4.6575</v>
+      </c>
+      <c r="J25" t="n">
+        <v>34.7016</v>
+      </c>
+      <c r="K25" t="n">
         <v>13.2171</v>
       </c>
-      <c r="J25" t="n">
+      <c r="L25" t="n">
         <v>38.5272</v>
       </c>
     </row>
@@ -1664,9 +1818,15 @@
         </is>
       </c>
       <c r="I26" t="n">
+        <v>7.6707</v>
+      </c>
+      <c r="J26" t="n">
+        <v>36.9238</v>
+      </c>
+      <c r="K26" t="n">
         <v>16.8582</v>
       </c>
-      <c r="J26" t="n">
+      <c r="L26" t="n">
         <v>30.6789</v>
       </c>
     </row>
@@ -1712,9 +1872,15 @@
         </is>
       </c>
       <c r="I27" t="n">
+        <v>8.161799999999999</v>
+      </c>
+      <c r="J27" t="n">
+        <v>36.9985</v>
+      </c>
+      <c r="K27" t="n">
         <v>19.3344</v>
       </c>
-      <c r="J27" t="n">
+      <c r="L27" t="n">
         <v>43.0702</v>
       </c>
     </row>
@@ -1760,9 +1926,15 @@
         </is>
       </c>
       <c r="I28" t="n">
+        <v>8.116099999999999</v>
+      </c>
+      <c r="J28" t="n">
+        <v>37.0757</v>
+      </c>
+      <c r="K28" t="n">
         <v>0.3583</v>
       </c>
-      <c r="J28" t="n">
+      <c r="L28" t="n">
         <v>35.924</v>
       </c>
     </row>
@@ -1808,9 +1980,15 @@
         </is>
       </c>
       <c r="I29" t="n">
+        <v>4.7449</v>
+      </c>
+      <c r="J29" t="n">
+        <v>35.1894</v>
+      </c>
+      <c r="K29" t="n">
         <v>16.2626</v>
       </c>
-      <c r="J29" t="n">
+      <c r="L29" t="n">
         <v>39.2512</v>
       </c>
     </row>
@@ -1856,9 +2034,15 @@
         </is>
       </c>
       <c r="I30" t="n">
+        <v>11.284</v>
+      </c>
+      <c r="J30" t="n">
+        <v>38.9047</v>
+      </c>
+      <c r="K30" t="n">
         <v>3.816</v>
       </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>42.2395</v>
       </c>
     </row>
@@ -1904,9 +2088,15 @@
         </is>
       </c>
       <c r="I31" t="n">
+        <v>10.8907</v>
+      </c>
+      <c r="J31" t="n">
+        <v>39.1093</v>
+      </c>
+      <c r="K31" t="n">
         <v>17.1638</v>
       </c>
-      <c r="J31" t="n">
+      <c r="L31" t="n">
         <v>38.0787</v>
       </c>
     </row>
@@ -1952,9 +2142,15 @@
         </is>
       </c>
       <c r="I32" t="n">
+        <v>5.3388</v>
+      </c>
+      <c r="J32" t="n">
+        <v>35.132</v>
+      </c>
+      <c r="K32" t="n">
         <v>14.052</v>
       </c>
-      <c r="J32" t="n">
+      <c r="L32" t="n">
         <v>44.458</v>
       </c>
     </row>
@@ -2000,9 +2196,15 @@
         </is>
       </c>
       <c r="I33" t="n">
+        <v>8.329000000000001</v>
+      </c>
+      <c r="J33" t="n">
+        <v>36.8436</v>
+      </c>
+      <c r="K33" t="n">
         <v>0.1575</v>
       </c>
-      <c r="J33" t="n">
+      <c r="L33" t="n">
         <v>39.4561</v>
       </c>
     </row>
@@ -2048,9 +2250,15 @@
         </is>
       </c>
       <c r="I34" t="n">
+        <v>11.1672</v>
+      </c>
+      <c r="J34" t="n">
+        <v>38.7224</v>
+      </c>
+      <c r="K34" t="n">
         <v>7.9936</v>
       </c>
-      <c r="J34" t="n">
+      <c r="L34" t="n">
         <v>37.7003</v>
       </c>
     </row>
@@ -2096,9 +2304,15 @@
         </is>
       </c>
       <c r="I35" t="n">
+        <v>11.1671</v>
+      </c>
+      <c r="J35" t="n">
+        <v>38.7442</v>
+      </c>
+      <c r="K35" t="n">
         <v>11.5281</v>
       </c>
-      <c r="J35" t="n">
+      <c r="L35" t="n">
         <v>38.2988</v>
       </c>
     </row>
@@ -2144,9 +2358,15 @@
         </is>
       </c>
       <c r="I36" t="n">
+        <v>8.2296</v>
+      </c>
+      <c r="J36" t="n">
+        <v>37.0039</v>
+      </c>
+      <c r="K36" t="n">
         <v>8.724600000000001</v>
       </c>
-      <c r="J36" t="n">
+      <c r="L36" t="n">
         <v>32.42</v>
       </c>
     </row>
@@ -2192,9 +2412,15 @@
         </is>
       </c>
       <c r="I37" t="n">
+        <v>11.0744</v>
+      </c>
+      <c r="J37" t="n">
+        <v>39.1057</v>
+      </c>
+      <c r="K37" t="n">
         <v>17.6635</v>
       </c>
-      <c r="J37" t="n">
+      <c r="L37" t="n">
         <v>40.8449</v>
       </c>
     </row>
@@ -2240,9 +2466,15 @@
         </is>
       </c>
       <c r="I38" t="n">
+        <v>8.103899999999999</v>
+      </c>
+      <c r="J38" t="n">
+        <v>37.2115</v>
+      </c>
+      <c r="K38" t="n">
         <v>4.1442</v>
       </c>
-      <c r="J38" t="n">
+      <c r="L38" t="n">
         <v>40.3605</v>
       </c>
     </row>
@@ -2288,9 +2520,15 @@
         </is>
       </c>
       <c r="I39" t="n">
+        <v>5.1079</v>
+      </c>
+      <c r="J39" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="K39" t="n">
         <v>6.073</v>
       </c>
-      <c r="J39" t="n">
+      <c r="L39" t="n">
         <v>33.1415</v>
       </c>
     </row>
@@ -2336,9 +2574,15 @@
         </is>
       </c>
       <c r="I40" t="n">
+        <v>4.6908</v>
+      </c>
+      <c r="J40" t="n">
+        <v>35.2439</v>
+      </c>
+      <c r="K40" t="n">
         <v>6.7547</v>
       </c>
-      <c r="J40" t="n">
+      <c r="L40" t="n">
         <v>31.7095</v>
       </c>
     </row>
@@ -2384,9 +2628,15 @@
         </is>
       </c>
       <c r="I41" t="n">
+        <v>8.226800000000001</v>
+      </c>
+      <c r="J41" t="n">
+        <v>37.3378</v>
+      </c>
+      <c r="K41" t="n">
         <v>17.0682</v>
       </c>
-      <c r="J41" t="n">
+      <c r="L41" t="n">
         <v>43.1054</v>
       </c>
     </row>
@@ -2432,9 +2682,15 @@
         </is>
       </c>
       <c r="I42" t="n">
+        <v>11.2736</v>
+      </c>
+      <c r="J42" t="n">
+        <v>39.2512</v>
+      </c>
+      <c r="K42" t="n">
         <v>12.1931</v>
       </c>
-      <c r="J42" t="n">
+      <c r="L42" t="n">
         <v>42.8758</v>
       </c>
     </row>
@@ -2480,9 +2736,15 @@
         </is>
       </c>
       <c r="I43" t="n">
+        <v>4.7956</v>
+      </c>
+      <c r="J43" t="n">
+        <v>35.0094</v>
+      </c>
+      <c r="K43" t="n">
         <v>14.567</v>
       </c>
-      <c r="J43" t="n">
+      <c r="L43" t="n">
         <v>40.6225</v>
       </c>
     </row>
@@ -2528,9 +2790,15 @@
         </is>
       </c>
       <c r="I44" t="n">
+        <v>14.1715</v>
+      </c>
+      <c r="J44" t="n">
+        <v>41.1981</v>
+      </c>
+      <c r="K44" t="n">
         <v>16.9719</v>
       </c>
-      <c r="J44" t="n">
+      <c r="L44" t="n">
         <v>36.5866</v>
       </c>
     </row>
@@ -2576,9 +2844,15 @@
         </is>
       </c>
       <c r="I45" t="n">
+        <v>7.8371</v>
+      </c>
+      <c r="J45" t="n">
+        <v>36.8098</v>
+      </c>
+      <c r="K45" t="n">
         <v>5.3203</v>
       </c>
-      <c r="J45" t="n">
+      <c r="L45" t="n">
         <v>40.728</v>
       </c>
     </row>
@@ -2624,9 +2898,15 @@
         </is>
       </c>
       <c r="I46" t="n">
+        <v>8.128399999999999</v>
+      </c>
+      <c r="J46" t="n">
+        <v>36.9958</v>
+      </c>
+      <c r="K46" t="n">
         <v>16.0354</v>
       </c>
-      <c r="J46" t="n">
+      <c r="L46" t="n">
         <v>36.2011</v>
       </c>
     </row>
@@ -2672,9 +2952,15 @@
         </is>
       </c>
       <c r="I47" t="n">
+        <v>8.218400000000001</v>
+      </c>
+      <c r="J47" t="n">
+        <v>36.9907</v>
+      </c>
+      <c r="K47" t="n">
         <v>15.403</v>
       </c>
-      <c r="J47" t="n">
+      <c r="L47" t="n">
         <v>40.7644</v>
       </c>
     </row>
@@ -2720,9 +3006,15 @@
         </is>
       </c>
       <c r="I48" t="n">
+        <v>11.3257</v>
+      </c>
+      <c r="J48" t="n">
+        <v>39.0236</v>
+      </c>
+      <c r="K48" t="n">
         <v>15.1838</v>
       </c>
-      <c r="J48" t="n">
+      <c r="L48" t="n">
         <v>39.9026</v>
       </c>
     </row>
@@ -2768,9 +3060,15 @@
         </is>
       </c>
       <c r="I49" t="n">
+        <v>11.1595</v>
+      </c>
+      <c r="J49" t="n">
+        <v>38.9749</v>
+      </c>
+      <c r="K49" t="n">
         <v>17.7157</v>
       </c>
-      <c r="J49" t="n">
+      <c r="L49" t="n">
         <v>40.5119</v>
       </c>
     </row>
@@ -2816,9 +3114,15 @@
         </is>
       </c>
       <c r="I50" t="n">
+        <v>16.7766</v>
+      </c>
+      <c r="J50" t="n">
+        <v>42.6601</v>
+      </c>
+      <c r="K50" t="n">
         <v>12.8776</v>
       </c>
-      <c r="J50" t="n">
+      <c r="L50" t="n">
         <v>43.3137</v>
       </c>
     </row>
@@ -2864,9 +3168,15 @@
         </is>
       </c>
       <c r="I51" t="n">
+        <v>10.8559</v>
+      </c>
+      <c r="J51" t="n">
+        <v>39.344</v>
+      </c>
+      <c r="K51" t="n">
         <v>1.6856</v>
       </c>
-      <c r="J51" t="n">
+      <c r="L51" t="n">
         <v>38.0615</v>
       </c>
     </row>
@@ -2912,9 +3222,15 @@
         </is>
       </c>
       <c r="I52" t="n">
+        <v>8.105</v>
+      </c>
+      <c r="J52" t="n">
+        <v>36.9335</v>
+      </c>
+      <c r="K52" t="n">
         <v>10.2334</v>
       </c>
-      <c r="J52" t="n">
+      <c r="L52" t="n">
         <v>34.6838</v>
       </c>
     </row>
@@ -2960,9 +3276,15 @@
         </is>
       </c>
       <c r="I53" t="n">
+        <v>7.9071</v>
+      </c>
+      <c r="J53" t="n">
+        <v>37.0572</v>
+      </c>
+      <c r="K53" t="n">
         <v>14.5302</v>
       </c>
-      <c r="J53" t="n">
+      <c r="L53" t="n">
         <v>44.8043</v>
       </c>
     </row>
@@ -3008,9 +3330,15 @@
         </is>
       </c>
       <c r="I54" t="n">
+        <v>4.9274</v>
+      </c>
+      <c r="J54" t="n">
+        <v>34.7603</v>
+      </c>
+      <c r="K54" t="n">
         <v>18.8269</v>
       </c>
-      <c r="J54" t="n">
+      <c r="L54" t="n">
         <v>36.7311</v>
       </c>
     </row>
@@ -3056,9 +3384,15 @@
         </is>
       </c>
       <c r="I55" t="n">
+        <v>10.7032</v>
+      </c>
+      <c r="J55" t="n">
+        <v>38.7757</v>
+      </c>
+      <c r="K55" t="n">
         <v>5.6907</v>
       </c>
-      <c r="J55" t="n">
+      <c r="L55" t="n">
         <v>41.7718</v>
       </c>
     </row>
@@ -3104,9 +3438,15 @@
         </is>
       </c>
       <c r="I56" t="n">
+        <v>11.2805</v>
+      </c>
+      <c r="J56" t="n">
+        <v>39.2196</v>
+      </c>
+      <c r="K56" t="n">
         <v>11.6474</v>
       </c>
-      <c r="J56" t="n">
+      <c r="L56" t="n">
         <v>42.3426</v>
       </c>
     </row>
@@ -3152,9 +3492,15 @@
         </is>
       </c>
       <c r="I57" t="n">
+        <v>8.0578</v>
+      </c>
+      <c r="J57" t="n">
+        <v>37.226</v>
+      </c>
+      <c r="K57" t="n">
         <v>17.7702</v>
       </c>
-      <c r="J57" t="n">
+      <c r="L57" t="n">
         <v>37.1438</v>
       </c>
     </row>
@@ -3200,9 +3546,15 @@
         </is>
       </c>
       <c r="I58" t="n">
+        <v>8.059200000000001</v>
+      </c>
+      <c r="J58" t="n">
+        <v>36.7697</v>
+      </c>
+      <c r="K58" t="n">
         <v>9.9765</v>
       </c>
-      <c r="J58" t="n">
+      <c r="L58" t="n">
         <v>36.3513</v>
       </c>
     </row>
@@ -3248,9 +3600,15 @@
         </is>
       </c>
       <c r="I59" t="n">
+        <v>7.8396</v>
+      </c>
+      <c r="J59" t="n">
+        <v>36.8372</v>
+      </c>
+      <c r="K59" t="n">
         <v>14.223</v>
       </c>
-      <c r="J59" t="n">
+      <c r="L59" t="n">
         <v>31.9408</v>
       </c>
     </row>
@@ -3296,9 +3654,15 @@
         </is>
       </c>
       <c r="I60" t="n">
+        <v>11.0251</v>
+      </c>
+      <c r="J60" t="n">
+        <v>39.2075</v>
+      </c>
+      <c r="K60" t="n">
         <v>7.3866</v>
       </c>
-      <c r="J60" t="n">
+      <c r="L60" t="n">
         <v>44.2773</v>
       </c>
     </row>
@@ -3344,9 +3708,15 @@
         </is>
       </c>
       <c r="I61" t="n">
+        <v>10.6999</v>
+      </c>
+      <c r="J61" t="n">
+        <v>39.1547</v>
+      </c>
+      <c r="K61" t="n">
         <v>6.0985</v>
       </c>
-      <c r="J61" t="n">
+      <c r="L61" t="n">
         <v>35.6169</v>
       </c>
     </row>
@@ -3392,9 +3762,15 @@
         </is>
       </c>
       <c r="I62" t="n">
+        <v>8.206200000000001</v>
+      </c>
+      <c r="J62" t="n">
+        <v>37.0288</v>
+      </c>
+      <c r="K62" t="n">
         <v>4.3116</v>
       </c>
-      <c r="J62" t="n">
+      <c r="L62" t="n">
         <v>42.2869</v>
       </c>
     </row>
@@ -3440,9 +3816,15 @@
         </is>
       </c>
       <c r="I63" t="n">
+        <v>10.9516</v>
+      </c>
+      <c r="J63" t="n">
+        <v>39.0337</v>
+      </c>
+      <c r="K63" t="n">
         <v>9.047499999999999</v>
       </c>
-      <c r="J63" t="n">
+      <c r="L63" t="n">
         <v>35.0673</v>
       </c>
     </row>
@@ -3488,9 +3870,15 @@
         </is>
       </c>
       <c r="I64" t="n">
+        <v>8.2155</v>
+      </c>
+      <c r="J64" t="n">
+        <v>36.7982</v>
+      </c>
+      <c r="K64" t="n">
         <v>8.9815</v>
       </c>
-      <c r="J64" t="n">
+      <c r="L64" t="n">
         <v>42.9952</v>
       </c>
     </row>
@@ -3536,9 +3924,15 @@
         </is>
       </c>
       <c r="I65" t="n">
+        <v>7.7406</v>
+      </c>
+      <c r="J65" t="n">
+        <v>37.3045</v>
+      </c>
+      <c r="K65" t="n">
         <v>0.9164</v>
       </c>
-      <c r="J65" t="n">
+      <c r="L65" t="n">
         <v>40.0567</v>
       </c>
     </row>
@@ -3584,9 +3978,15 @@
         </is>
       </c>
       <c r="I66" t="n">
+        <v>7.696</v>
+      </c>
+      <c r="J66" t="n">
+        <v>37.1135</v>
+      </c>
+      <c r="K66" t="n">
         <v>11.1871</v>
       </c>
-      <c r="J66" t="n">
+      <c r="L66" t="n">
         <v>32.8864</v>
       </c>
     </row>
@@ -3632,9 +4032,15 @@
         </is>
       </c>
       <c r="I67" t="n">
+        <v>10.9452</v>
+      </c>
+      <c r="J67" t="n">
+        <v>38.8969</v>
+      </c>
+      <c r="K67" t="n">
         <v>13.1651</v>
       </c>
-      <c r="J67" t="n">
+      <c r="L67" t="n">
         <v>37.9779</v>
       </c>
     </row>
@@ -3680,9 +4086,15 @@
         </is>
       </c>
       <c r="I68" t="n">
+        <v>16.8799</v>
+      </c>
+      <c r="J68" t="n">
+        <v>43.1493</v>
+      </c>
+      <c r="K68" t="n">
         <v>12.1371</v>
       </c>
-      <c r="J68" t="n">
+      <c r="L68" t="n">
         <v>36.027</v>
       </c>
     </row>
@@ -3728,9 +4140,15 @@
         </is>
       </c>
       <c r="I69" t="n">
+        <v>5.1485</v>
+      </c>
+      <c r="J69" t="n">
+        <v>35.2102</v>
+      </c>
+      <c r="K69" t="n">
         <v>5.1436</v>
       </c>
-      <c r="J69" t="n">
+      <c r="L69" t="n">
         <v>31.7197</v>
       </c>
     </row>
@@ -3776,9 +4194,15 @@
         </is>
       </c>
       <c r="I70" t="n">
+        <v>5.0515</v>
+      </c>
+      <c r="J70" t="n">
+        <v>34.67</v>
+      </c>
+      <c r="K70" t="n">
         <v>13.5722</v>
       </c>
-      <c r="J70" t="n">
+      <c r="L70" t="n">
         <v>30.8837</v>
       </c>
     </row>
@@ -3824,9 +4248,15 @@
         </is>
       </c>
       <c r="I71" t="n">
+        <v>16.7522</v>
+      </c>
+      <c r="J71" t="n">
+        <v>43.1062</v>
+      </c>
+      <c r="K71" t="n">
         <v>17.8602</v>
       </c>
-      <c r="J71" t="n">
+      <c r="L71" t="n">
         <v>33.869</v>
       </c>
     </row>
@@ -3872,9 +4302,15 @@
         </is>
       </c>
       <c r="I72" t="n">
+        <v>16.8931</v>
+      </c>
+      <c r="J72" t="n">
+        <v>42.7009</v>
+      </c>
+      <c r="K72" t="n">
         <v>15.0478</v>
       </c>
-      <c r="J72" t="n">
+      <c r="L72" t="n">
         <v>35.7757</v>
       </c>
     </row>
@@ -3920,9 +4356,15 @@
         </is>
       </c>
       <c r="I73" t="n">
+        <v>4.7326</v>
+      </c>
+      <c r="J73" t="n">
+        <v>34.696</v>
+      </c>
+      <c r="K73" t="n">
         <v>4.6748</v>
       </c>
-      <c r="J73" t="n">
+      <c r="L73" t="n">
         <v>43.2923</v>
       </c>
     </row>
@@ -3968,9 +4410,15 @@
         </is>
       </c>
       <c r="I74" t="n">
+        <v>7.7538</v>
+      </c>
+      <c r="J74" t="n">
+        <v>36.7034</v>
+      </c>
+      <c r="K74" t="n">
         <v>8.1349</v>
       </c>
-      <c r="J74" t="n">
+      <c r="L74" t="n">
         <v>31.2586</v>
       </c>
     </row>
@@ -4016,9 +4464,15 @@
         </is>
       </c>
       <c r="I75" t="n">
+        <v>10.8418</v>
+      </c>
+      <c r="J75" t="n">
+        <v>38.8872</v>
+      </c>
+      <c r="K75" t="n">
         <v>9.034800000000001</v>
       </c>
-      <c r="J75" t="n">
+      <c r="L75" t="n">
         <v>30.015</v>
       </c>
     </row>
@@ -4064,9 +4518,15 @@
         </is>
       </c>
       <c r="I76" t="n">
+        <v>7.7152</v>
+      </c>
+      <c r="J76" t="n">
+        <v>36.9925</v>
+      </c>
+      <c r="K76" t="n">
         <v>11.9574</v>
       </c>
-      <c r="J76" t="n">
+      <c r="L76" t="n">
         <v>42.5923</v>
       </c>
     </row>
@@ -4112,9 +4572,15 @@
         </is>
       </c>
       <c r="I77" t="n">
+        <v>7.8742</v>
+      </c>
+      <c r="J77" t="n">
+        <v>37.0614</v>
+      </c>
+      <c r="K77" t="n">
         <v>14.7837</v>
       </c>
-      <c r="J77" t="n">
+      <c r="L77" t="n">
         <v>38.4462</v>
       </c>
     </row>
@@ -4160,9 +4626,15 @@
         </is>
       </c>
       <c r="I78" t="n">
+        <v>8.2888</v>
+      </c>
+      <c r="J78" t="n">
+        <v>37.0946</v>
+      </c>
+      <c r="K78" t="n">
         <v>12.2089</v>
       </c>
-      <c r="J78" t="n">
+      <c r="L78" t="n">
         <v>44.3613</v>
       </c>
     </row>
@@ -4208,9 +4680,15 @@
         </is>
       </c>
       <c r="I79" t="n">
+        <v>7.6564</v>
+      </c>
+      <c r="J79" t="n">
+        <v>36.9237</v>
+      </c>
+      <c r="K79" t="n">
         <v>13.2455</v>
       </c>
-      <c r="J79" t="n">
+      <c r="L79" t="n">
         <v>34.8246</v>
       </c>
     </row>
@@ -4256,9 +4734,15 @@
         </is>
       </c>
       <c r="I80" t="n">
+        <v>8.157999999999999</v>
+      </c>
+      <c r="J80" t="n">
+        <v>37.1958</v>
+      </c>
+      <c r="K80" t="n">
         <v>18.0289</v>
       </c>
-      <c r="J80" t="n">
+      <c r="L80" t="n">
         <v>40.0906</v>
       </c>
     </row>
@@ -4304,9 +4788,15 @@
         </is>
       </c>
       <c r="I81" t="n">
+        <v>8.051299999999999</v>
+      </c>
+      <c r="J81" t="n">
+        <v>36.8542</v>
+      </c>
+      <c r="K81" t="n">
         <v>0.619</v>
       </c>
-      <c r="J81" t="n">
+      <c r="L81" t="n">
         <v>42.4813</v>
       </c>
     </row>
@@ -4352,9 +4842,15 @@
         </is>
       </c>
       <c r="I82" t="n">
+        <v>11.0304</v>
+      </c>
+      <c r="J82" t="n">
+        <v>39.2614</v>
+      </c>
+      <c r="K82" t="n">
         <v>16.7829</v>
       </c>
-      <c r="J82" t="n">
+      <c r="L82" t="n">
         <v>42.178</v>
       </c>
     </row>
@@ -4400,9 +4896,15 @@
         </is>
       </c>
       <c r="I83" t="n">
+        <v>3.3288</v>
+      </c>
+      <c r="J83" t="n">
+        <v>32.8397</v>
+      </c>
+      <c r="K83" t="n">
         <v>13.6111</v>
       </c>
-      <c r="J83" t="n">
+      <c r="L83" t="n">
         <v>40.638</v>
       </c>
     </row>
@@ -4448,9 +4950,15 @@
         </is>
       </c>
       <c r="I84" t="n">
+        <v>8.1883</v>
+      </c>
+      <c r="J84" t="n">
+        <v>37.2388</v>
+      </c>
+      <c r="K84" t="n">
         <v>0.7359</v>
       </c>
-      <c r="J84" t="n">
+      <c r="L84" t="n">
         <v>37.3926</v>
       </c>
     </row>
@@ -4496,9 +5004,15 @@
         </is>
       </c>
       <c r="I85" t="n">
+        <v>10.8407</v>
+      </c>
+      <c r="J85" t="n">
+        <v>38.6984</v>
+      </c>
+      <c r="K85" t="n">
         <v>11.382</v>
       </c>
-      <c r="J85" t="n">
+      <c r="L85" t="n">
         <v>37.4102</v>
       </c>
     </row>
@@ -4544,9 +5058,15 @@
         </is>
       </c>
       <c r="I86" t="n">
+        <v>10.821</v>
+      </c>
+      <c r="J86" t="n">
+        <v>38.69</v>
+      </c>
+      <c r="K86" t="n">
         <v>2.5649</v>
       </c>
-      <c r="J86" t="n">
+      <c r="L86" t="n">
         <v>30.9757</v>
       </c>
     </row>
@@ -4592,9 +5112,15 @@
         </is>
       </c>
       <c r="I87" t="n">
+        <v>8.212400000000001</v>
+      </c>
+      <c r="J87" t="n">
+        <v>36.9458</v>
+      </c>
+      <c r="K87" t="n">
         <v>13.5547</v>
       </c>
-      <c r="J87" t="n">
+      <c r="L87" t="n">
         <v>39.2168</v>
       </c>
     </row>
@@ -4640,9 +5166,15 @@
         </is>
       </c>
       <c r="I88" t="n">
+        <v>10.8669</v>
+      </c>
+      <c r="J88" t="n">
+        <v>38.7778</v>
+      </c>
+      <c r="K88" t="n">
         <v>16.8868</v>
       </c>
-      <c r="J88" t="n">
+      <c r="L88" t="n">
         <v>36.1031</v>
       </c>
     </row>
@@ -4688,9 +5220,15 @@
         </is>
       </c>
       <c r="I89" t="n">
+        <v>4.9661</v>
+      </c>
+      <c r="J89" t="n">
+        <v>35.2064</v>
+      </c>
+      <c r="K89" t="n">
         <v>18.3678</v>
       </c>
-      <c r="J89" t="n">
+      <c r="L89" t="n">
         <v>37.9862</v>
       </c>
     </row>
@@ -4736,9 +5274,15 @@
         </is>
       </c>
       <c r="I90" t="n">
+        <v>7.6829</v>
+      </c>
+      <c r="J90" t="n">
+        <v>36.9176</v>
+      </c>
+      <c r="K90" t="n">
         <v>18.3399</v>
       </c>
-      <c r="J90" t="n">
+      <c r="L90" t="n">
         <v>32.9532</v>
       </c>
     </row>
@@ -4784,9 +5328,15 @@
         </is>
       </c>
       <c r="I91" t="n">
+        <v>8.1021</v>
+      </c>
+      <c r="J91" t="n">
+        <v>37.267</v>
+      </c>
+      <c r="K91" t="n">
         <v>4.9431</v>
       </c>
-      <c r="J91" t="n">
+      <c r="L91" t="n">
         <v>37.1036</v>
       </c>
     </row>

</xml_diff>